<commit_message>
Replace app with sanitized desktop 1.1 source
</commit_message>
<xml_diff>
--- a/templates/quotation-reference.xlsx
+++ b/templates/quotation-reference.xlsx
@@ -7,10 +7,15 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Quotation Layout" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Quotation" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Calculation" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Price List" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cost &amp; Margin" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Notes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Quotation Layout'!$8:$8</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Quotation'!$8:$8</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Calculation'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -18,8 +23,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="6">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="&quot;RM&quot;#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+  </numFmts>
+  <fonts count="22">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,24 +37,94 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <color rgb="00595959"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <b val="1"/>
       <sz val="13"/>
+    </font>
+    <font>
+      <sz val="8.5"/>
     </font>
     <font>
       <b val="1"/>
       <sz val="9"/>
     </font>
     <font>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="00000000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <color rgb="00000000"/>
       <sz val="8.5"/>
     </font>
     <font>
-      <sz val="9"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="14"/>
     </font>
     <font>
-      <b val="1"/>
-      <sz val="12"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -55,11 +133,36 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF9E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E2F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00EDEDED"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF3FE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -74,18 +177,66 @@
       <right style="thin">
         <color rgb="00BFBFBF"/>
       </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
       <top style="medium">
         <color rgb="00000000"/>
       </top>
       <bottom style="thin">
         <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00000000"/>
       </bottom>
     </border>
     <border>
       <left/>
       <right/>
-      <top style="medium">
-        <color rgb="00000000"/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
       </top>
       <bottom style="thin">
         <color rgb="00BFBFBF"/>
@@ -97,11 +248,35 @@
       <right style="thin">
         <color rgb="00BFBFBF"/>
       </right>
-      <top style="medium">
-        <color rgb="00000000"/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
       </top>
       <bottom style="thin">
         <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00000000"/>
       </bottom>
       <diagonal/>
     </border>
@@ -125,38 +300,162 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="medium">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -520,9 +819,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.5" customWidth="1" min="1" max="1"/>
@@ -559,42 +858,1490 @@
     </row>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="7" t="n"/>
-      <c r="B7" s="8" t="n"/>
-      <c r="C7" s="8" t="n"/>
-      <c r="D7" s="8" t="n"/>
-      <c r="E7" s="8" t="n"/>
-      <c r="F7" s="8" t="n"/>
-      <c r="G7" s="8" t="n"/>
-      <c r="H7" s="8" t="n"/>
-      <c r="I7" s="8" t="n"/>
-      <c r="J7" s="9" t="n"/>
+      <c r="B7" s="53" t="n"/>
+      <c r="C7" s="53" t="n"/>
+      <c r="D7" s="53" t="n"/>
+      <c r="E7" s="53" t="n"/>
+      <c r="F7" s="53" t="n"/>
+      <c r="G7" s="53" t="n"/>
+      <c r="H7" s="53" t="n"/>
+      <c r="I7" s="53" t="n"/>
+      <c r="J7" s="54" t="n"/>
     </row>
     <row r="8" ht="44" customHeight="1">
-      <c r="A8" s="10" t="n"/>
-      <c r="B8" s="10" t="n"/>
-      <c r="C8" s="10" t="n"/>
-      <c r="D8" s="10" t="n"/>
-      <c r="E8" s="10" t="n"/>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="10" t="n"/>
-      <c r="H8" s="10" t="n"/>
-      <c r="I8" s="10" t="n"/>
-      <c r="J8" s="10" t="n"/>
+      <c r="A8" s="9" t="n"/>
+      <c r="B8" s="9" t="n"/>
+      <c r="C8" s="9" t="n"/>
+      <c r="D8" s="9" t="n"/>
+      <c r="E8" s="9" t="n"/>
+      <c r="F8" s="9" t="n"/>
+      <c r="G8" s="9" t="n"/>
+      <c r="H8" s="9" t="n"/>
+      <c r="I8" s="9" t="n"/>
+      <c r="J8" s="9" t="n"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="10" t="n"/>
+      <c r="B9" s="55" t="n"/>
+      <c r="C9" s="55" t="n"/>
+      <c r="D9" s="55" t="n"/>
+      <c r="E9" s="55" t="n"/>
+      <c r="F9" s="55" t="n"/>
+      <c r="G9" s="55" t="n"/>
+      <c r="H9" s="55" t="n"/>
+      <c r="I9" s="55" t="n"/>
+      <c r="J9" s="56" t="n"/>
+    </row>
+    <row r="10" ht="97" customHeight="1">
+      <c r="A10" s="12" t="n"/>
+      <c r="B10" s="13" t="n"/>
+      <c r="C10" s="12" t="n"/>
+      <c r="D10" s="13" t="n"/>
+      <c r="E10" s="12" t="n"/>
+      <c r="F10" s="14" t="n"/>
+      <c r="G10" s="12" t="n"/>
+      <c r="H10" s="15" t="n"/>
+      <c r="I10" s="16" t="n"/>
+      <c r="J10" s="17" t="n"/>
+    </row>
+    <row r="11" ht="97" customHeight="1">
+      <c r="A11" s="12" t="n"/>
+      <c r="B11" s="13" t="n"/>
+      <c r="C11" s="12" t="n"/>
+      <c r="D11" s="13" t="n"/>
+      <c r="E11" s="12" t="n"/>
+      <c r="F11" s="14" t="n"/>
+      <c r="G11" s="12" t="n"/>
+      <c r="H11" s="15" t="n"/>
+      <c r="I11" s="16" t="n"/>
+      <c r="J11" s="17" t="n"/>
+    </row>
+    <row r="12" ht="97" customHeight="1">
+      <c r="A12" s="12" t="n"/>
+      <c r="B12" s="13" t="n"/>
+      <c r="C12" s="12" t="n"/>
+      <c r="D12" s="13" t="n"/>
+      <c r="E12" s="12" t="n"/>
+      <c r="F12" s="14" t="n"/>
+      <c r="G12" s="12" t="n"/>
+      <c r="H12" s="15" t="n"/>
+      <c r="I12" s="16" t="n"/>
+      <c r="J12" s="17" t="n"/>
+    </row>
+    <row r="13" ht="97" customHeight="1">
+      <c r="A13" s="12" t="n"/>
+      <c r="B13" s="13" t="n"/>
+      <c r="C13" s="12" t="n"/>
+      <c r="D13" s="13" t="n"/>
+      <c r="E13" s="12" t="n"/>
+      <c r="F13" s="14" t="n"/>
+      <c r="G13" s="12" t="n"/>
+      <c r="H13" s="15" t="n"/>
+      <c r="I13" s="16" t="n"/>
+      <c r="J13" s="17" t="n"/>
+    </row>
+    <row r="14" ht="97" customHeight="1">
+      <c r="A14" s="12" t="n"/>
+      <c r="B14" s="13" t="n"/>
+      <c r="C14" s="12" t="n"/>
+      <c r="D14" s="13" t="n"/>
+      <c r="E14" s="12" t="n"/>
+      <c r="F14" s="14" t="n"/>
+      <c r="G14" s="12" t="n"/>
+      <c r="H14" s="15" t="n"/>
+      <c r="I14" s="16" t="n"/>
+      <c r="J14" s="17" t="n"/>
+    </row>
+    <row r="15" ht="97" customHeight="1">
+      <c r="A15" s="12" t="n"/>
+      <c r="B15" s="13" t="n"/>
+      <c r="C15" s="12" t="n"/>
+      <c r="D15" s="13" t="n"/>
+      <c r="E15" s="12" t="n"/>
+      <c r="F15" s="14" t="n"/>
+      <c r="G15" s="12" t="n"/>
+      <c r="H15" s="15" t="n"/>
+      <c r="I15" s="16" t="n"/>
+      <c r="J15" s="17" t="n"/>
+    </row>
+    <row r="16" ht="97" customHeight="1">
+      <c r="A16" s="12" t="n"/>
+      <c r="B16" s="13" t="n"/>
+      <c r="C16" s="12" t="n"/>
+      <c r="D16" s="13" t="n"/>
+      <c r="E16" s="12" t="n"/>
+      <c r="F16" s="14" t="n"/>
+      <c r="G16" s="12" t="n"/>
+      <c r="H16" s="15" t="n"/>
+      <c r="I16" s="16" t="n"/>
+      <c r="J16" s="17" t="n"/>
+    </row>
+    <row r="17" ht="97" customHeight="1">
+      <c r="A17" s="12" t="n"/>
+      <c r="B17" s="13" t="n"/>
+      <c r="C17" s="12" t="n"/>
+      <c r="D17" s="13" t="n"/>
+      <c r="E17" s="12" t="n"/>
+      <c r="F17" s="14" t="n"/>
+      <c r="G17" s="12" t="n"/>
+      <c r="H17" s="15" t="n"/>
+      <c r="I17" s="16" t="n"/>
+      <c r="J17" s="17" t="n"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="10" t="n"/>
+      <c r="B18" s="55" t="n"/>
+      <c r="C18" s="55" t="n"/>
+      <c r="D18" s="55" t="n"/>
+      <c r="E18" s="55" t="n"/>
+      <c r="F18" s="55" t="n"/>
+      <c r="G18" s="55" t="n"/>
+      <c r="H18" s="55" t="n"/>
+      <c r="I18" s="55" t="n"/>
+      <c r="J18" s="56" t="n"/>
+    </row>
+    <row r="19" ht="97" customHeight="1">
+      <c r="A19" s="12" t="n"/>
+      <c r="B19" s="13" t="n"/>
+      <c r="C19" s="12" t="n"/>
+      <c r="D19" s="13" t="n"/>
+      <c r="E19" s="12" t="n"/>
+      <c r="F19" s="14" t="n"/>
+      <c r="G19" s="12" t="n"/>
+      <c r="H19" s="15" t="n"/>
+      <c r="I19" s="16" t="n"/>
+      <c r="J19" s="17" t="n"/>
+    </row>
+    <row r="20" ht="97" customHeight="1">
+      <c r="A20" s="12" t="n"/>
+      <c r="B20" s="13" t="n"/>
+      <c r="C20" s="12" t="n"/>
+      <c r="D20" s="13" t="n"/>
+      <c r="E20" s="12" t="n"/>
+      <c r="F20" s="14" t="n"/>
+      <c r="G20" s="12" t="n"/>
+      <c r="H20" s="15" t="n"/>
+      <c r="I20" s="16" t="n"/>
+      <c r="J20" s="17" t="n"/>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="18" t="n"/>
+      <c r="B21" s="57" t="n"/>
+      <c r="C21" s="57" t="n"/>
+      <c r="D21" s="57" t="n"/>
+      <c r="E21" s="57" t="n"/>
+      <c r="F21" s="57" t="n"/>
+      <c r="G21" s="57" t="n"/>
+      <c r="H21" s="58" t="n"/>
+      <c r="I21" s="20" t="n"/>
+      <c r="J21" s="19" t="n"/>
+    </row>
+    <row r="22" ht="16" customHeight="1">
+      <c r="A22" s="21" t="n"/>
+    </row>
+    <row r="23"/>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="22" t="n"/>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="23" t="n"/>
+    </row>
+    <row r="26" ht="31" customHeight="1">
+      <c r="A26" s="23" t="n"/>
+    </row>
+    <row r="27" ht="31" customHeight="1">
+      <c r="A27" s="23" t="n"/>
+    </row>
+    <row r="28" ht="31" customHeight="1">
+      <c r="A28" s="23" t="n"/>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="23" t="n"/>
+    </row>
+    <row r="30"/>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="22" t="n"/>
+    </row>
+    <row r="32" ht="44" customHeight="1">
+      <c r="A32" s="24" t="n"/>
+    </row>
+    <row r="33" ht="44" customHeight="1">
+      <c r="A33" s="24" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="21">
     <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A32:J32"/>
+    <mergeCell ref="A22:J22"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="A29:J29"/>
+    <mergeCell ref="A28:J28"/>
     <mergeCell ref="C2:H2"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="A21:H21"/>
     <mergeCell ref="A6:J6"/>
-    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="C3:H3"/>
+    <mergeCell ref="A25:J25"/>
+    <mergeCell ref="I1:J1"/>
+    <mergeCell ref="A18:J18"/>
+    <mergeCell ref="A27:J27"/>
     <mergeCell ref="A1:B4"/>
-    <mergeCell ref="A7:J7"/>
     <mergeCell ref="C4:H4"/>
-    <mergeCell ref="C3:H3"/>
-    <mergeCell ref="I1:J1"/>
+    <mergeCell ref="A26:J26"/>
+    <mergeCell ref="A33:J33"/>
     <mergeCell ref="C1:H1"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:Y27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="14" max="14"/>
+    <col width="6" customWidth="1" min="15" max="15"/>
+    <col width="7" customWidth="1" min="16" max="16"/>
+    <col width="11" customWidth="1" min="17" max="17"/>
+    <col width="6" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="56" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="26" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="25" t="n"/>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="26" t="n"/>
+    </row>
+    <row r="3" ht="40" customHeight="1">
+      <c r="A3" s="26" t="n"/>
+    </row>
+    <row r="4" ht="46" customHeight="1">
+      <c r="A4" s="27" t="n"/>
+      <c r="B4" s="27" t="n"/>
+      <c r="C4" s="27" t="n"/>
+      <c r="D4" s="27" t="n"/>
+      <c r="E4" s="27" t="n"/>
+      <c r="F4" s="27" t="n"/>
+      <c r="G4" s="27" t="n"/>
+      <c r="H4" s="27" t="n"/>
+      <c r="I4" s="27" t="n"/>
+      <c r="J4" s="27" t="n"/>
+      <c r="K4" s="27" t="n"/>
+      <c r="L4" s="27" t="n"/>
+      <c r="M4" s="27" t="n"/>
+      <c r="N4" s="27" t="n"/>
+      <c r="O4" s="27" t="n"/>
+      <c r="P4" s="27" t="n"/>
+      <c r="Q4" s="27" t="n"/>
+      <c r="R4" s="27" t="n"/>
+      <c r="S4" s="27" t="n"/>
+      <c r="T4" s="27" t="n"/>
+      <c r="U4" s="27" t="n"/>
+      <c r="V4" s="27" t="n"/>
+      <c r="W4" s="27" t="n"/>
+      <c r="X4" s="27" t="n"/>
+      <c r="Y4" s="27" t="n"/>
+    </row>
+    <row r="5" ht="42" customHeight="1">
+      <c r="A5" s="12" t="n"/>
+      <c r="B5" s="13" t="n"/>
+      <c r="C5" s="13" t="n"/>
+      <c r="D5" s="13" t="n"/>
+      <c r="E5" s="13" t="n"/>
+      <c r="F5" s="13" t="n"/>
+      <c r="G5" s="28" t="n"/>
+      <c r="H5" s="28" t="n"/>
+      <c r="I5" s="28" t="n"/>
+      <c r="J5" s="14" t="n"/>
+      <c r="K5" s="14" t="n"/>
+      <c r="L5" s="14" t="n"/>
+      <c r="M5" s="14" t="n"/>
+      <c r="N5" s="14" t="n"/>
+      <c r="O5" s="12" t="n"/>
+      <c r="P5" s="14" t="n"/>
+      <c r="Q5" s="16" t="n"/>
+      <c r="R5" s="15" t="n"/>
+      <c r="S5" s="29" t="n"/>
+      <c r="T5" s="13" t="n"/>
+      <c r="U5" s="16" t="n"/>
+      <c r="V5" s="13" t="n"/>
+      <c r="W5" s="16" t="n"/>
+      <c r="X5" s="16" t="n"/>
+      <c r="Y5" s="13" t="n"/>
+    </row>
+    <row r="6" ht="42" customHeight="1">
+      <c r="A6" s="12" t="n"/>
+      <c r="B6" s="13" t="n"/>
+      <c r="C6" s="13" t="n"/>
+      <c r="D6" s="13" t="n"/>
+      <c r="E6" s="13" t="n"/>
+      <c r="F6" s="13" t="n"/>
+      <c r="G6" s="28" t="n"/>
+      <c r="H6" s="28" t="n"/>
+      <c r="I6" s="28" t="n"/>
+      <c r="J6" s="14" t="n"/>
+      <c r="K6" s="14" t="n"/>
+      <c r="L6" s="14" t="n"/>
+      <c r="M6" s="14" t="n"/>
+      <c r="N6" s="14" t="n"/>
+      <c r="O6" s="12" t="n"/>
+      <c r="P6" s="14" t="n"/>
+      <c r="Q6" s="16" t="n"/>
+      <c r="R6" s="15" t="n"/>
+      <c r="S6" s="29" t="n"/>
+      <c r="T6" s="13" t="n"/>
+      <c r="U6" s="16" t="n"/>
+      <c r="V6" s="13" t="n"/>
+      <c r="W6" s="16" t="n"/>
+      <c r="X6" s="16" t="n"/>
+      <c r="Y6" s="13" t="n"/>
+    </row>
+    <row r="7" ht="42" customHeight="1">
+      <c r="A7" s="12" t="n"/>
+      <c r="B7" s="13" t="n"/>
+      <c r="C7" s="13" t="n"/>
+      <c r="D7" s="13" t="n"/>
+      <c r="E7" s="13" t="n"/>
+      <c r="F7" s="13" t="n"/>
+      <c r="G7" s="28" t="n"/>
+      <c r="H7" s="28" t="n"/>
+      <c r="I7" s="28" t="n"/>
+      <c r="J7" s="14" t="n"/>
+      <c r="K7" s="14" t="n"/>
+      <c r="L7" s="14" t="n"/>
+      <c r="M7" s="14" t="n"/>
+      <c r="N7" s="14" t="n"/>
+      <c r="O7" s="12" t="n"/>
+      <c r="P7" s="14" t="n"/>
+      <c r="Q7" s="16" t="n"/>
+      <c r="R7" s="15" t="n"/>
+      <c r="S7" s="29" t="n"/>
+      <c r="T7" s="13" t="n"/>
+      <c r="U7" s="16" t="n"/>
+      <c r="V7" s="13" t="n"/>
+      <c r="W7" s="16" t="n"/>
+      <c r="X7" s="16" t="n"/>
+      <c r="Y7" s="13" t="n"/>
+    </row>
+    <row r="8" ht="42" customHeight="1">
+      <c r="A8" s="12" t="n"/>
+      <c r="B8" s="13" t="n"/>
+      <c r="C8" s="13" t="n"/>
+      <c r="D8" s="13" t="n"/>
+      <c r="E8" s="13" t="n"/>
+      <c r="F8" s="13" t="n"/>
+      <c r="G8" s="28" t="n"/>
+      <c r="H8" s="28" t="n"/>
+      <c r="I8" s="28" t="n"/>
+      <c r="J8" s="14" t="n"/>
+      <c r="K8" s="14" t="n"/>
+      <c r="L8" s="14" t="n"/>
+      <c r="M8" s="14" t="n"/>
+      <c r="N8" s="14" t="n"/>
+      <c r="O8" s="12" t="n"/>
+      <c r="P8" s="14" t="n"/>
+      <c r="Q8" s="16" t="n"/>
+      <c r="R8" s="15" t="n"/>
+      <c r="S8" s="29" t="n"/>
+      <c r="T8" s="13" t="n"/>
+      <c r="U8" s="16" t="n"/>
+      <c r="V8" s="13" t="n"/>
+      <c r="W8" s="16" t="n"/>
+      <c r="X8" s="16" t="n"/>
+      <c r="Y8" s="13" t="n"/>
+    </row>
+    <row r="9" ht="42" customHeight="1">
+      <c r="A9" s="12" t="n"/>
+      <c r="B9" s="13" t="n"/>
+      <c r="C9" s="13" t="n"/>
+      <c r="D9" s="13" t="n"/>
+      <c r="E9" s="13" t="n"/>
+      <c r="F9" s="13" t="n"/>
+      <c r="G9" s="28" t="n"/>
+      <c r="H9" s="28" t="n"/>
+      <c r="I9" s="28" t="n"/>
+      <c r="J9" s="14" t="n"/>
+      <c r="K9" s="14" t="n"/>
+      <c r="L9" s="14" t="n"/>
+      <c r="M9" s="14" t="n"/>
+      <c r="N9" s="14" t="n"/>
+      <c r="O9" s="12" t="n"/>
+      <c r="P9" s="14" t="n"/>
+      <c r="Q9" s="16" t="n"/>
+      <c r="R9" s="15" t="n"/>
+      <c r="S9" s="29" t="n"/>
+      <c r="T9" s="13" t="n"/>
+      <c r="U9" s="16" t="n"/>
+      <c r="V9" s="13" t="n"/>
+      <c r="W9" s="16" t="n"/>
+      <c r="X9" s="16" t="n"/>
+      <c r="Y9" s="13" t="n"/>
+    </row>
+    <row r="10" ht="42" customHeight="1">
+      <c r="A10" s="12" t="n"/>
+      <c r="B10" s="13" t="n"/>
+      <c r="C10" s="13" t="n"/>
+      <c r="D10" s="13" t="n"/>
+      <c r="E10" s="13" t="n"/>
+      <c r="F10" s="13" t="n"/>
+      <c r="G10" s="28" t="n"/>
+      <c r="H10" s="28" t="n"/>
+      <c r="I10" s="28" t="n"/>
+      <c r="J10" s="14" t="n"/>
+      <c r="K10" s="14" t="n"/>
+      <c r="L10" s="14" t="n"/>
+      <c r="M10" s="14" t="n"/>
+      <c r="N10" s="14" t="n"/>
+      <c r="O10" s="12" t="n"/>
+      <c r="P10" s="14" t="n"/>
+      <c r="Q10" s="16" t="n"/>
+      <c r="R10" s="15" t="n"/>
+      <c r="S10" s="29" t="n"/>
+      <c r="T10" s="13" t="n"/>
+      <c r="U10" s="16" t="n"/>
+      <c r="V10" s="13" t="n"/>
+      <c r="W10" s="16" t="n"/>
+      <c r="X10" s="16" t="n"/>
+      <c r="Y10" s="13" t="n"/>
+    </row>
+    <row r="11" ht="42" customHeight="1">
+      <c r="A11" s="12" t="n"/>
+      <c r="B11" s="13" t="n"/>
+      <c r="C11" s="13" t="n"/>
+      <c r="D11" s="13" t="n"/>
+      <c r="E11" s="13" t="n"/>
+      <c r="F11" s="13" t="n"/>
+      <c r="G11" s="28" t="n"/>
+      <c r="H11" s="28" t="n"/>
+      <c r="I11" s="28" t="n"/>
+      <c r="J11" s="14" t="n"/>
+      <c r="K11" s="14" t="n"/>
+      <c r="L11" s="14" t="n"/>
+      <c r="M11" s="14" t="n"/>
+      <c r="N11" s="14" t="n"/>
+      <c r="O11" s="12" t="n"/>
+      <c r="P11" s="14" t="n"/>
+      <c r="Q11" s="16" t="n"/>
+      <c r="R11" s="15" t="n"/>
+      <c r="S11" s="29" t="n"/>
+      <c r="T11" s="13" t="n"/>
+      <c r="U11" s="16" t="n"/>
+      <c r="V11" s="13" t="n"/>
+      <c r="W11" s="16" t="n"/>
+      <c r="X11" s="16" t="n"/>
+      <c r="Y11" s="13" t="n"/>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="12" t="n"/>
+      <c r="B12" s="13" t="n"/>
+      <c r="C12" s="13" t="n"/>
+      <c r="D12" s="13" t="n"/>
+      <c r="E12" s="13" t="n"/>
+      <c r="F12" s="13" t="n"/>
+      <c r="G12" s="28" t="n"/>
+      <c r="H12" s="28" t="n"/>
+      <c r="I12" s="28" t="n"/>
+      <c r="J12" s="14" t="n"/>
+      <c r="K12" s="14" t="n"/>
+      <c r="L12" s="14" t="n"/>
+      <c r="M12" s="14" t="n"/>
+      <c r="N12" s="14" t="n"/>
+      <c r="O12" s="12" t="n"/>
+      <c r="P12" s="14" t="n"/>
+      <c r="Q12" s="16" t="n"/>
+      <c r="R12" s="15" t="n"/>
+      <c r="S12" s="29" t="n"/>
+      <c r="T12" s="13" t="n"/>
+      <c r="U12" s="16" t="n"/>
+      <c r="V12" s="13" t="n"/>
+      <c r="W12" s="16" t="n"/>
+      <c r="X12" s="16" t="n"/>
+      <c r="Y12" s="13" t="n"/>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="A13" s="12" t="n"/>
+      <c r="B13" s="13" t="n"/>
+      <c r="C13" s="13" t="n"/>
+      <c r="D13" s="13" t="n"/>
+      <c r="E13" s="13" t="n"/>
+      <c r="F13" s="13" t="n"/>
+      <c r="G13" s="28" t="n"/>
+      <c r="H13" s="28" t="n"/>
+      <c r="I13" s="28" t="n"/>
+      <c r="J13" s="14" t="n"/>
+      <c r="K13" s="14" t="n"/>
+      <c r="L13" s="14" t="n"/>
+      <c r="M13" s="14" t="n"/>
+      <c r="N13" s="14" t="n"/>
+      <c r="O13" s="12" t="n"/>
+      <c r="P13" s="14" t="n"/>
+      <c r="Q13" s="16" t="n"/>
+      <c r="R13" s="15" t="n"/>
+      <c r="S13" s="29" t="n"/>
+      <c r="T13" s="13" t="n"/>
+      <c r="U13" s="16" t="n"/>
+      <c r="V13" s="13" t="n"/>
+      <c r="W13" s="16" t="n"/>
+      <c r="X13" s="16" t="n"/>
+      <c r="Y13" s="13" t="n"/>
+    </row>
+    <row r="14" ht="42" customHeight="1">
+      <c r="A14" s="12" t="n"/>
+      <c r="B14" s="13" t="n"/>
+      <c r="C14" s="13" t="n"/>
+      <c r="D14" s="13" t="n"/>
+      <c r="E14" s="13" t="n"/>
+      <c r="F14" s="13" t="n"/>
+      <c r="G14" s="28" t="n"/>
+      <c r="H14" s="28" t="n"/>
+      <c r="I14" s="28" t="n"/>
+      <c r="J14" s="14" t="n"/>
+      <c r="K14" s="14" t="n"/>
+      <c r="L14" s="14" t="n"/>
+      <c r="M14" s="14" t="n"/>
+      <c r="N14" s="14" t="n"/>
+      <c r="O14" s="12" t="n"/>
+      <c r="P14" s="14" t="n"/>
+      <c r="Q14" s="16" t="n"/>
+      <c r="R14" s="15" t="n"/>
+      <c r="S14" s="29" t="n"/>
+      <c r="T14" s="13" t="n"/>
+      <c r="U14" s="16" t="n"/>
+      <c r="V14" s="13" t="n"/>
+      <c r="W14" s="16" t="n"/>
+      <c r="X14" s="16" t="n"/>
+      <c r="Y14" s="13" t="n"/>
+    </row>
+    <row r="15"/>
+    <row r="16">
+      <c r="A16" s="30" t="n"/>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="31" t="n"/>
+      <c r="S17" s="32" t="n"/>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="31" t="n"/>
+      <c r="S18" s="32" t="n"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="33" t="n"/>
+      <c r="S19" s="34" t="n"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="33" t="n"/>
+      <c r="S20" s="34" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="35" t="n"/>
+      <c r="B21" s="55" t="n"/>
+      <c r="C21" s="55" t="n"/>
+      <c r="D21" s="55" t="n"/>
+      <c r="E21" s="55" t="n"/>
+      <c r="F21" s="55" t="n"/>
+      <c r="G21" s="55" t="n"/>
+      <c r="H21" s="55" t="n"/>
+      <c r="I21" s="55" t="n"/>
+      <c r="J21" s="55" t="n"/>
+      <c r="K21" s="55" t="n"/>
+      <c r="L21" s="55" t="n"/>
+      <c r="M21" s="55" t="n"/>
+      <c r="N21" s="55" t="n"/>
+      <c r="O21" s="55" t="n"/>
+      <c r="P21" s="55" t="n"/>
+      <c r="Q21" s="55" t="n"/>
+      <c r="R21" s="56" t="n"/>
+      <c r="S21" s="37" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="38" t="n"/>
+      <c r="S22" s="39" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="35" t="n"/>
+      <c r="B23" s="55" t="n"/>
+      <c r="C23" s="55" t="n"/>
+      <c r="D23" s="55" t="n"/>
+      <c r="E23" s="55" t="n"/>
+      <c r="F23" s="55" t="n"/>
+      <c r="G23" s="55" t="n"/>
+      <c r="H23" s="55" t="n"/>
+      <c r="I23" s="55" t="n"/>
+      <c r="J23" s="55" t="n"/>
+      <c r="K23" s="55" t="n"/>
+      <c r="L23" s="55" t="n"/>
+      <c r="M23" s="55" t="n"/>
+      <c r="N23" s="55" t="n"/>
+      <c r="O23" s="55" t="n"/>
+      <c r="P23" s="55" t="n"/>
+      <c r="Q23" s="55" t="n"/>
+      <c r="R23" s="56" t="n"/>
+      <c r="S23" s="40" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="38" t="n"/>
+      <c r="S24" s="41" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="38" t="n"/>
+      <c r="S25" s="42" t="n"/>
+    </row>
+    <row r="26"/>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="21" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="A16:V16"/>
+    <mergeCell ref="A20:R20"/>
+    <mergeCell ref="A21:R21"/>
+    <mergeCell ref="A2:Y2"/>
+    <mergeCell ref="A25:R25"/>
+    <mergeCell ref="A24:R24"/>
+    <mergeCell ref="A19:R19"/>
+    <mergeCell ref="A1:Y1"/>
+    <mergeCell ref="A27:V27"/>
+    <mergeCell ref="A17:R17"/>
+    <mergeCell ref="A23:R23"/>
+    <mergeCell ref="A3:Y3"/>
+    <mergeCell ref="A22:R22"/>
+    <mergeCell ref="A18:R18"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:L11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="52" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="43" t="n"/>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="33" t="n"/>
+    </row>
+    <row r="3" ht="46" customHeight="1">
+      <c r="A3" s="27" t="n"/>
+      <c r="B3" s="27" t="n"/>
+      <c r="C3" s="27" t="n"/>
+      <c r="D3" s="27" t="n"/>
+      <c r="E3" s="27" t="n"/>
+      <c r="F3" s="27" t="n"/>
+      <c r="G3" s="27" t="n"/>
+      <c r="H3" s="27" t="n"/>
+      <c r="I3" s="27" t="n"/>
+      <c r="J3" s="27" t="n"/>
+      <c r="K3" s="27" t="n"/>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="13" t="n"/>
+      <c r="B4" s="13" t="n"/>
+      <c r="C4" s="13" t="n"/>
+      <c r="D4" s="16" t="n"/>
+      <c r="E4" s="16" t="n"/>
+      <c r="F4" s="16" t="n"/>
+      <c r="G4" s="16" t="n"/>
+      <c r="H4" s="44" t="n"/>
+      <c r="I4" s="12" t="n"/>
+      <c r="J4" s="12" t="n"/>
+      <c r="K4" s="13" t="n"/>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="13" t="n"/>
+      <c r="B5" s="13" t="n"/>
+      <c r="C5" s="13" t="n"/>
+      <c r="D5" s="16" t="n"/>
+      <c r="E5" s="16" t="n"/>
+      <c r="F5" s="16" t="n"/>
+      <c r="G5" s="16" t="n"/>
+      <c r="H5" s="44" t="n"/>
+      <c r="I5" s="12" t="n"/>
+      <c r="J5" s="12" t="n"/>
+      <c r="K5" s="13" t="n"/>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="13" t="n"/>
+      <c r="B6" s="13" t="n"/>
+      <c r="C6" s="13" t="n"/>
+      <c r="D6" s="16" t="n"/>
+      <c r="E6" s="16" t="n"/>
+      <c r="F6" s="16" t="n"/>
+      <c r="G6" s="16" t="n"/>
+      <c r="H6" s="44" t="n"/>
+      <c r="I6" s="12" t="n"/>
+      <c r="J6" s="12" t="n"/>
+      <c r="K6" s="13" t="n"/>
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="13" t="n"/>
+      <c r="B7" s="13" t="n"/>
+      <c r="C7" s="13" t="n"/>
+      <c r="D7" s="16" t="n"/>
+      <c r="E7" s="16" t="n"/>
+      <c r="F7" s="16" t="n"/>
+      <c r="G7" s="16" t="n"/>
+      <c r="H7" s="44" t="n"/>
+      <c r="I7" s="12" t="n"/>
+      <c r="J7" s="12" t="n"/>
+      <c r="K7" s="13" t="n"/>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="13" t="n"/>
+      <c r="B8" s="13" t="n"/>
+      <c r="C8" s="13" t="n"/>
+      <c r="D8" s="16" t="n"/>
+      <c r="E8" s="16" t="n"/>
+      <c r="F8" s="16" t="n"/>
+      <c r="G8" s="16" t="n"/>
+      <c r="H8" s="44" t="n"/>
+      <c r="I8" s="12" t="n"/>
+      <c r="J8" s="12" t="n"/>
+      <c r="K8" s="13" t="n"/>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="13" t="n"/>
+      <c r="B9" s="13" t="n"/>
+      <c r="C9" s="13" t="n"/>
+      <c r="D9" s="16" t="n"/>
+      <c r="E9" s="16" t="n"/>
+      <c r="F9" s="16" t="n"/>
+      <c r="G9" s="16" t="n"/>
+      <c r="H9" s="44" t="n"/>
+      <c r="I9" s="12" t="n"/>
+      <c r="J9" s="12" t="n"/>
+      <c r="K9" s="13" t="n"/>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="13" t="n"/>
+      <c r="B10" s="13" t="n"/>
+      <c r="C10" s="13" t="n"/>
+      <c r="D10" s="16" t="n"/>
+      <c r="E10" s="16" t="n"/>
+      <c r="F10" s="16" t="n"/>
+      <c r="G10" s="16" t="n"/>
+      <c r="H10" s="44" t="n"/>
+      <c r="I10" s="12" t="n"/>
+      <c r="J10" s="12" t="n"/>
+      <c r="K10" s="13" t="n"/>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="13" t="n"/>
+      <c r="B11" s="13" t="n"/>
+      <c r="C11" s="13" t="n"/>
+      <c r="D11" s="16" t="n"/>
+      <c r="E11" s="16" t="n"/>
+      <c r="F11" s="16" t="n"/>
+      <c r="G11" s="16" t="n"/>
+      <c r="H11" s="44" t="n"/>
+      <c r="I11" s="12" t="n"/>
+      <c r="J11" s="12" t="n"/>
+      <c r="K11" s="13" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A1:K1"/>
+  </mergeCells>
+  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:L14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="45" t="n"/>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="33" t="n"/>
+    </row>
+    <row r="3" ht="46" customHeight="1">
+      <c r="A3" s="27" t="n"/>
+      <c r="B3" s="27" t="n"/>
+      <c r="C3" s="27" t="n"/>
+      <c r="D3" s="27" t="n"/>
+      <c r="E3" s="27" t="n"/>
+      <c r="F3" s="27" t="n"/>
+      <c r="G3" s="27" t="n"/>
+      <c r="H3" s="27" t="n"/>
+      <c r="I3" s="27" t="n"/>
+      <c r="J3" s="27" t="n"/>
+      <c r="K3" s="27" t="n"/>
+      <c r="L3" s="27" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="12" t="n"/>
+      <c r="B4" s="13" t="n"/>
+      <c r="C4" s="13" t="n"/>
+      <c r="D4" s="14" t="n"/>
+      <c r="E4" s="14" t="n"/>
+      <c r="F4" s="15" t="n"/>
+      <c r="G4" s="16" t="n"/>
+      <c r="H4" s="16" t="n"/>
+      <c r="I4" s="16" t="n"/>
+      <c r="J4" s="16" t="n"/>
+      <c r="K4" s="46" t="n"/>
+      <c r="L4" s="13" t="n"/>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="12" t="n"/>
+      <c r="B5" s="13" t="n"/>
+      <c r="C5" s="13" t="n"/>
+      <c r="D5" s="14" t="n"/>
+      <c r="E5" s="14" t="n"/>
+      <c r="F5" s="15" t="n"/>
+      <c r="G5" s="16" t="n"/>
+      <c r="H5" s="16" t="n"/>
+      <c r="I5" s="16" t="n"/>
+      <c r="J5" s="16" t="n"/>
+      <c r="K5" s="46" t="n"/>
+      <c r="L5" s="13" t="n"/>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="12" t="n"/>
+      <c r="B6" s="13" t="n"/>
+      <c r="C6" s="13" t="n"/>
+      <c r="D6" s="14" t="n"/>
+      <c r="E6" s="14" t="n"/>
+      <c r="F6" s="15" t="n"/>
+      <c r="G6" s="16" t="n"/>
+      <c r="H6" s="16" t="n"/>
+      <c r="I6" s="16" t="n"/>
+      <c r="J6" s="16" t="n"/>
+      <c r="K6" s="46" t="n"/>
+      <c r="L6" s="13" t="n"/>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="12" t="n"/>
+      <c r="B7" s="13" t="n"/>
+      <c r="C7" s="13" t="n"/>
+      <c r="D7" s="14" t="n"/>
+      <c r="E7" s="14" t="n"/>
+      <c r="F7" s="15" t="n"/>
+      <c r="G7" s="16" t="n"/>
+      <c r="H7" s="16" t="n"/>
+      <c r="I7" s="16" t="n"/>
+      <c r="J7" s="16" t="n"/>
+      <c r="K7" s="46" t="n"/>
+      <c r="L7" s="13" t="n"/>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="12" t="n"/>
+      <c r="B8" s="13" t="n"/>
+      <c r="C8" s="13" t="n"/>
+      <c r="D8" s="14" t="n"/>
+      <c r="E8" s="14" t="n"/>
+      <c r="F8" s="15" t="n"/>
+      <c r="G8" s="16" t="n"/>
+      <c r="H8" s="16" t="n"/>
+      <c r="I8" s="16" t="n"/>
+      <c r="J8" s="16" t="n"/>
+      <c r="K8" s="46" t="n"/>
+      <c r="L8" s="13" t="n"/>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="12" t="n"/>
+      <c r="B9" s="13" t="n"/>
+      <c r="C9" s="13" t="n"/>
+      <c r="D9" s="14" t="n"/>
+      <c r="E9" s="14" t="n"/>
+      <c r="F9" s="15" t="n"/>
+      <c r="G9" s="16" t="n"/>
+      <c r="H9" s="16" t="n"/>
+      <c r="I9" s="16" t="n"/>
+      <c r="J9" s="16" t="n"/>
+      <c r="K9" s="46" t="n"/>
+      <c r="L9" s="13" t="n"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="12" t="n"/>
+      <c r="B10" s="13" t="n"/>
+      <c r="C10" s="13" t="n"/>
+      <c r="D10" s="14" t="n"/>
+      <c r="E10" s="14" t="n"/>
+      <c r="F10" s="15" t="n"/>
+      <c r="G10" s="16" t="n"/>
+      <c r="H10" s="16" t="n"/>
+      <c r="I10" s="16" t="n"/>
+      <c r="J10" s="16" t="n"/>
+      <c r="K10" s="46" t="n"/>
+      <c r="L10" s="13" t="n"/>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="12" t="n"/>
+      <c r="B11" s="13" t="n"/>
+      <c r="C11" s="13" t="n"/>
+      <c r="D11" s="14" t="n"/>
+      <c r="E11" s="14" t="n"/>
+      <c r="F11" s="15" t="n"/>
+      <c r="G11" s="16" t="n"/>
+      <c r="H11" s="16" t="n"/>
+      <c r="I11" s="16" t="n"/>
+      <c r="J11" s="16" t="n"/>
+      <c r="K11" s="46" t="n"/>
+      <c r="L11" s="13" t="n"/>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="12" t="n"/>
+      <c r="B12" s="13" t="n"/>
+      <c r="C12" s="13" t="n"/>
+      <c r="D12" s="14" t="n"/>
+      <c r="E12" s="14" t="n"/>
+      <c r="F12" s="15" t="n"/>
+      <c r="G12" s="16" t="n"/>
+      <c r="H12" s="16" t="n"/>
+      <c r="I12" s="16" t="n"/>
+      <c r="J12" s="16" t="n"/>
+      <c r="K12" s="46" t="n"/>
+      <c r="L12" s="13" t="n"/>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="12" t="n"/>
+      <c r="B13" s="13" t="n"/>
+      <c r="C13" s="13" t="n"/>
+      <c r="D13" s="14" t="n"/>
+      <c r="E13" s="14" t="n"/>
+      <c r="F13" s="15" t="n"/>
+      <c r="G13" s="16" t="n"/>
+      <c r="H13" s="16" t="n"/>
+      <c r="I13" s="16" t="n"/>
+      <c r="J13" s="16" t="n"/>
+      <c r="K13" s="46" t="n"/>
+      <c r="L13" s="13" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="47" t="n"/>
+      <c r="B14" s="55" t="n"/>
+      <c r="C14" s="55" t="n"/>
+      <c r="D14" s="55" t="n"/>
+      <c r="E14" s="55" t="n"/>
+      <c r="F14" s="55" t="n"/>
+      <c r="G14" s="56" t="n"/>
+      <c r="H14" s="48" t="n"/>
+      <c r="I14" s="48" t="n"/>
+      <c r="J14" s="48" t="n"/>
+      <c r="K14" s="49" t="n"/>
+      <c r="L14" s="36" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A1:L1"/>
+  </mergeCells>
+  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:F111"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="130" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="50" t="n"/>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="51" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="52" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="52" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="52" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="52" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="52" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="52" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="52" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="52" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="52" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="52" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="52" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="52" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="52" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="52" t="n"/>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" s="51" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="52" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="52" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="52" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="52" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="52" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="52" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="52" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="52" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="52" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="52" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="52" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="52" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="52" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="52" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="52" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="52" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="52" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="52" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="52" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="52" t="n"/>
+    </row>
+    <row r="40"/>
+    <row r="41">
+      <c r="A41" s="51" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="52" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="52" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="52" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="52" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="52" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="52" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="52" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="52" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="52" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="52" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="52" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="52" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="52" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="52" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="52" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="52" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="52" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="52" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="52" t="n"/>
+    </row>
+    <row r="61"/>
+    <row r="62">
+      <c r="A62" s="51" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="52" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="52" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="52" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="52" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="52" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="52" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="52" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="52" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="52" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="52" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="52" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="52" t="n"/>
+    </row>
+    <row r="75"/>
+    <row r="76">
+      <c r="A76" s="51" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="52" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="52" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="52" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="52" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="52" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="52" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="52" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="52" t="n"/>
+    </row>
+    <row r="85"/>
+    <row r="86">
+      <c r="A86" s="51" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="52" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="52" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="52" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="52" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="52" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="52" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="52" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="52" t="n"/>
+    </row>
+    <row r="95"/>
+    <row r="96">
+      <c r="A96" s="51" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="52" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="52" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="52" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="52" t="n"/>
+    </row>
+    <row r="101"/>
+    <row r="102">
+      <c r="A102" s="51" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="52" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="52" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="52" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="52" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="52" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="52" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="52" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="52" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="52" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="103">
+    <mergeCell ref="A84:F84"/>
+    <mergeCell ref="A66:F66"/>
+    <mergeCell ref="A50:F50"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A55:F55"/>
+    <mergeCell ref="A86:F86"/>
+    <mergeCell ref="A47:F47"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A32:F32"/>
+    <mergeCell ref="A97:F97"/>
+    <mergeCell ref="A20:F20"/>
+    <mergeCell ref="A72:F72"/>
+    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A81:F81"/>
+    <mergeCell ref="A38:F38"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A44:F44"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A58:F58"/>
+    <mergeCell ref="A15:F15"/>
+    <mergeCell ref="A64:F64"/>
+    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="A73:F73"/>
+    <mergeCell ref="A51:F51"/>
+    <mergeCell ref="A107:F107"/>
+    <mergeCell ref="A82:F82"/>
+    <mergeCell ref="A60:F60"/>
+    <mergeCell ref="A70:F70"/>
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="A41:F41"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A99:F99"/>
+    <mergeCell ref="A108:F108"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A42:F42"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A35:F35"/>
+    <mergeCell ref="A62:F62"/>
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="A48:F48"/>
+    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A59:F59"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A98:F98"/>
+    <mergeCell ref="A79:F79"/>
+    <mergeCell ref="A88:F88"/>
+    <mergeCell ref="A54:F54"/>
+    <mergeCell ref="A46:F46"/>
+    <mergeCell ref="A90:F90"/>
+    <mergeCell ref="A74:F74"/>
+    <mergeCell ref="A105:F105"/>
+    <mergeCell ref="A56:F56"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="A71:F71"/>
+    <mergeCell ref="A76:F76"/>
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A100:F100"/>
+    <mergeCell ref="A53:F53"/>
+    <mergeCell ref="A109:F109"/>
+    <mergeCell ref="A63:F63"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A93:F93"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A68:F68"/>
+    <mergeCell ref="A102:F102"/>
+    <mergeCell ref="A111:F111"/>
+    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="A83:F83"/>
+    <mergeCell ref="A92:F92"/>
+    <mergeCell ref="A39:F39"/>
+    <mergeCell ref="A49:F49"/>
+    <mergeCell ref="A36:F36"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A45:F45"/>
+    <mergeCell ref="A94:F94"/>
+    <mergeCell ref="A103:F103"/>
+    <mergeCell ref="A78:F78"/>
+    <mergeCell ref="A87:F87"/>
+    <mergeCell ref="A65:F65"/>
+    <mergeCell ref="A80:F80"/>
+    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="A89:F89"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="A104:F104"/>
+    <mergeCell ref="A57:F57"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A106:F106"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A96:F96"/>
+    <mergeCell ref="A91:F91"/>
+    <mergeCell ref="A43:F43"/>
+    <mergeCell ref="A52:F52"/>
+    <mergeCell ref="A67:F67"/>
+    <mergeCell ref="A77:F77"/>
+    <mergeCell ref="A110:F110"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A69:F69"/>
+    <mergeCell ref="A25:F25"/>
+  </mergeCells>
+  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>